<commit_message>
separação de classificação por sexo
</commit_message>
<xml_diff>
--- a/data_charge/planilha_modelo.xlsx
+++ b/data_charge/planilha_modelo.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29711"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0EABC2B-1A10-45AC-9EB4-CFEFA3F075AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\running_oab\running_classification\data_charge\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2722DC94-CE73-4BF2-A935-23170AD76EC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31275" yWindow="1665" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -22,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -31,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="50">
   <si>
     <t xml:space="preserve">NUMERO </t>
   </si>
@@ -178,6 +181,9 @@
   </si>
   <si>
     <t>60a99</t>
+  </si>
+  <si>
+    <t>IDADE</t>
   </si>
 </sst>
 </file>
@@ -187,7 +193,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -232,10 +238,10 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -259,7 +265,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -555,19 +561,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -575,434 +582,491 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="4">
+        <v>25</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>22</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="4">
+        <v>36</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>20</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="4">
+        <v>18</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="4">
+        <v>22</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>65</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="4">
+        <v>44</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>40</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="4">
+        <v>56</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>356</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="4">
+        <v>50</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="H8" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>342</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="4">
+        <v>60</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>500</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="4">
+        <v>62</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>45</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="4">
+        <v>46</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="F11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>654</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="4">
+        <v>29</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="H12" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>6522</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="4">
+        <v>30</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="H13" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>521</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="4">
+        <v>78</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="G14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="H14" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>501</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="4">
+        <v>45</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="G15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="H15" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="4">
+        <v>59</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="G16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="H16" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>481</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="4">
+        <v>32</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="H17" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>3001</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="4">
+        <v>49</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="G18" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="H18" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>171</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="4">
+        <v>63</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="4"/>
+      <c r="F19" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="G19" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="H19" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1010,6 +1074,7 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Alteração para possibilitar correção de registro
</commit_message>
<xml_diff>
--- a/data_charge/planilha_modelo.xlsx
+++ b/data_charge/planilha_modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\running_oab\running_classification\data_charge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB2D1B9-31E5-4DA7-887A-A00FF737C95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E39FE78D-AFE5-4A0F-9C6E-2783D72D61B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="31275" yWindow="1665" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="46">
   <si>
     <t xml:space="preserve">NUMERO </t>
   </si>
@@ -72,9 +72,6 @@
     <t>CAMBUÍ</t>
   </si>
   <si>
-    <t>18 a 29</t>
-  </si>
-  <si>
     <t>Sim</t>
   </si>
   <si>
@@ -90,9 +87,6 @@
     <t>CAMBUI</t>
   </si>
   <si>
-    <t>30 a 39</t>
-  </si>
-  <si>
     <t>FLAVIO ALEX DE CARVALHO</t>
   </si>
   <si>
@@ -108,9 +102,6 @@
     <t>ESTIVA</t>
   </si>
   <si>
-    <t>40 a 49</t>
-  </si>
-  <si>
     <t>JOSÉ APARECIDO</t>
   </si>
   <si>
@@ -123,9 +114,6 @@
     <t>POUSO ALEGRE</t>
   </si>
   <si>
-    <t>50 a 59</t>
-  </si>
-  <si>
     <t>RUDYNEI LAMIN</t>
   </si>
   <si>
@@ -183,10 +171,10 @@
     <t>Narnia</t>
   </si>
   <si>
-    <t>60a99</t>
-  </si>
-  <si>
     <t>IDADE</t>
+  </si>
+  <si>
+    <t>NÃO PREENCHER</t>
   </si>
 </sst>
 </file>
@@ -196,7 +184,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -216,6 +204,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -238,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -253,6 +249,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -567,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -576,7 +573,7 @@
     <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -588,7 +585,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -626,10 +623,10 @@
         <v>10</v>
       </c>
       <c r="G2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>12</v>
       </c>
       <c r="O2" s="4">
         <v>25</v>
@@ -640,25 +637,25 @@
         <v>22</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" s="5">
         <v>32875</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="G3" s="4" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O3" s="4">
         <v>36</v>
@@ -669,25 +666,25 @@
         <v>20</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C4" s="5">
         <v>39492</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="G4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>19</v>
       </c>
       <c r="O4" s="4">
         <v>18</v>
@@ -698,7 +695,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C5" s="5">
         <v>37996</v>
@@ -707,16 +704,16 @@
         <v>8</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O5" s="4">
         <v>22</v>
@@ -727,25 +724,25 @@
         <v>65</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C6" s="5">
         <v>30011</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G6" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>12</v>
       </c>
       <c r="O6" s="4">
         <v>44</v>
@@ -756,25 +753,25 @@
         <v>40</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C7" s="5">
         <v>25601</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O7" s="4">
         <v>56</v>
@@ -785,25 +782,25 @@
         <v>356</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C8" s="5">
         <v>27760</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O8" s="4">
         <v>50</v>
@@ -814,7 +811,7 @@
         <v>342</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C9" s="4">
         <v>60</v>
@@ -823,16 +820,16 @@
         <v>8</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O9" s="4">
         <v>60</v>
@@ -843,7 +840,7 @@
         <v>500</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C10" s="4">
         <v>62</v>
@@ -852,16 +849,16 @@
         <v>8</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O10" s="4">
         <v>62</v>
@@ -872,7 +869,7 @@
         <v>45</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C11" s="4">
         <v>46</v>
@@ -884,13 +881,13 @@
         <v>9</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O11" s="4">
         <v>46</v>
@@ -901,7 +898,7 @@
         <v>654</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C12" s="4">
         <v>29</v>
@@ -913,13 +910,13 @@
         <v>9</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O12" s="4">
         <v>29</v>
@@ -930,25 +927,25 @@
         <v>6522</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C13" s="4">
         <v>30</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O13" s="4">
         <v>30</v>
@@ -959,25 +956,25 @@
         <v>521</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C14" s="4">
         <v>78</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O14" s="4">
         <v>78</v>
@@ -988,25 +985,25 @@
         <v>501</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C15" s="4">
         <v>45</v>
       </c>
       <c r="D15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="G15" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>19</v>
       </c>
       <c r="O15" s="4">
         <v>45</v>
@@ -1017,25 +1014,25 @@
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C16" s="4">
         <v>59</v>
       </c>
       <c r="D16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="G16" s="4" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O16" s="4">
         <v>59</v>
@@ -1046,25 +1043,25 @@
         <v>481</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C17" s="4">
         <v>32</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E17" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="G17" s="4" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O17" s="4">
         <v>32</v>
@@ -1075,25 +1072,25 @@
         <v>3001</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C18" s="4">
         <v>49</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O18" s="4">
         <v>49</v>
@@ -1104,7 +1101,7 @@
         <v>171</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C19" s="4">
         <v>63</v>
@@ -1114,13 +1111,13 @@
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O19" s="4">
         <v>63</v>
@@ -1136,6 +1133,9 @@
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
     </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G21" s="6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
ajuste na geração de relatorio por categoria OAB
</commit_message>
<xml_diff>
--- a/data_charge/planilha_modelo.xlsx
+++ b/data_charge/planilha_modelo.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\running_oab\running_classification\data_charge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17C83F08-90FB-4048-84DB-2A0051B3CA09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D422A6-9543-45E8-973C-B526D335D98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26085" yWindow="2100" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
     <sheet name="Planilha2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$J$173</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -679,7 +679,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    <numFmt numFmtId="169" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -762,30 +762,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -805,13 +797,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1144,35 +1136,35 @@
     <col min="11" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="J1" s="12" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1183,7 +1175,7 @@
       <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="22">
+      <c r="C2" s="18">
         <v>26</v>
       </c>
       <c r="D2" s="3">
@@ -1192,18 +1184,18 @@
       <c r="E2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F2" s="17"/>
+      <c r="F2" s="13"/>
       <c r="G2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P2" s="17"/>
+      <c r="P2" s="13"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
@@ -1212,7 +1204,7 @@
       <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="18">
         <v>28</v>
       </c>
       <c r="D3" s="3">
@@ -1221,18 +1213,18 @@
       <c r="E3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="17"/>
+      <c r="F3" s="13"/>
       <c r="G3" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P3" s="17"/>
+      <c r="P3" s="13"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1241,7 +1233,7 @@
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="18">
         <v>26</v>
       </c>
       <c r="D4" s="3">
@@ -1250,18 +1242,18 @@
       <c r="E4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="17"/>
+      <c r="F4" s="13"/>
       <c r="G4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P4" s="17"/>
+      <c r="P4" s="13"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
@@ -1270,7 +1262,7 @@
       <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="18">
         <v>29</v>
       </c>
       <c r="D5" s="3">
@@ -1279,18 +1271,18 @@
       <c r="E5" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="17"/>
+      <c r="F5" s="13"/>
       <c r="G5" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P5" s="17"/>
+      <c r="P5" s="13"/>
     </row>
     <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1299,7 +1291,7 @@
       <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="23">
+      <c r="C6" s="19">
         <v>27</v>
       </c>
       <c r="D6" s="3">
@@ -1308,18 +1300,18 @@
       <c r="E6" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="17"/>
+      <c r="F6" s="13"/>
       <c r="G6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P6" s="17"/>
+      <c r="P6" s="13"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
@@ -1328,7 +1320,7 @@
       <c r="B7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="18">
         <v>27</v>
       </c>
       <c r="D7" s="3">
@@ -1337,18 +1329,18 @@
       <c r="E7" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="17"/>
+      <c r="F7" s="13"/>
       <c r="G7" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="17" t="s">
+      <c r="H7" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P7" s="17"/>
+      <c r="P7" s="13"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
@@ -1357,7 +1349,7 @@
       <c r="B8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="18">
         <v>28</v>
       </c>
       <c r="D8" s="3">
@@ -1366,18 +1358,18 @@
       <c r="E8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="17"/>
+      <c r="F8" s="13"/>
       <c r="G8" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="17" t="s">
+      <c r="H8" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P8" s="17"/>
+      <c r="P8" s="13"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -1386,7 +1378,7 @@
       <c r="B9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="18">
         <v>22</v>
       </c>
       <c r="D9" s="3">
@@ -1395,18 +1387,18 @@
       <c r="E9" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="17"/>
+      <c r="F9" s="13"/>
       <c r="G9" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H9" s="17" t="s">
+      <c r="H9" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P9" s="17"/>
+      <c r="P9" s="13"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
@@ -1415,7 +1407,7 @@
       <c r="B10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="18">
         <v>26</v>
       </c>
       <c r="D10" s="3">
@@ -1424,18 +1416,18 @@
       <c r="E10" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="17"/>
+      <c r="F10" s="13"/>
       <c r="G10" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H10" s="17" t="s">
+      <c r="H10" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P10" s="17"/>
+      <c r="P10" s="13"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
@@ -1444,7 +1436,7 @@
       <c r="B11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="18">
         <v>26</v>
       </c>
       <c r="D11" s="3">
@@ -1453,18 +1445,18 @@
       <c r="E11" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F11" s="17"/>
+      <c r="F11" s="13"/>
       <c r="G11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="H11" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P11" s="17"/>
+      <c r="P11" s="13"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
@@ -1473,7 +1465,7 @@
       <c r="B12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="18">
         <v>25</v>
       </c>
       <c r="D12" s="4">
@@ -1482,18 +1474,18 @@
       <c r="E12" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="17"/>
+      <c r="F12" s="13"/>
       <c r="G12" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H12" s="17" t="s">
+      <c r="H12" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P12" s="17"/>
+      <c r="P12" s="13"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
@@ -1502,7 +1494,7 @@
       <c r="B13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="18">
         <v>22</v>
       </c>
       <c r="D13" s="3">
@@ -1511,18 +1503,18 @@
       <c r="E13" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="17"/>
+      <c r="F13" s="13"/>
       <c r="G13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H13" s="17" t="s">
+      <c r="H13" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P13" s="17"/>
+      <c r="P13" s="13"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
@@ -1531,7 +1523,7 @@
       <c r="B14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="18">
         <v>24</v>
       </c>
       <c r="D14" s="4">
@@ -1540,18 +1532,18 @@
       <c r="E14" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="17"/>
+      <c r="F14" s="13"/>
       <c r="G14" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H14" s="17" t="s">
+      <c r="H14" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P14" s="17"/>
+      <c r="P14" s="13"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
@@ -1560,7 +1552,7 @@
       <c r="B15" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="18">
         <v>27</v>
       </c>
       <c r="D15" s="3">
@@ -1569,18 +1561,18 @@
       <c r="E15" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="17"/>
+      <c r="F15" s="13"/>
       <c r="G15" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H15" s="17" t="s">
+      <c r="H15" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P15" s="17"/>
+      <c r="P15" s="13"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
@@ -1589,7 +1581,7 @@
       <c r="B16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="18">
         <v>29</v>
       </c>
       <c r="D16" s="3">
@@ -1598,18 +1590,18 @@
       <c r="E16" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F16" s="17"/>
+      <c r="F16" s="13"/>
       <c r="G16" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H16" s="17" t="s">
+      <c r="H16" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P16" s="17"/>
+      <c r="P16" s="13"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
@@ -1618,7 +1610,7 @@
       <c r="B17" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="18">
         <v>28</v>
       </c>
       <c r="D17" s="3">
@@ -1627,18 +1619,18 @@
       <c r="E17" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F17" s="17"/>
+      <c r="F17" s="13"/>
       <c r="G17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P17" s="17"/>
+      <c r="P17" s="13"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
@@ -1647,7 +1639,7 @@
       <c r="B18" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="18">
         <v>27</v>
       </c>
       <c r="D18" s="3">
@@ -1656,18 +1648,18 @@
       <c r="E18" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F18" s="17"/>
+      <c r="F18" s="13"/>
       <c r="G18" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H18" s="17" t="s">
+      <c r="H18" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P18" s="17"/>
+      <c r="P18" s="13"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
@@ -1676,7 +1668,7 @@
       <c r="B19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="18">
         <v>27</v>
       </c>
       <c r="D19" s="3">
@@ -1685,18 +1677,18 @@
       <c r="E19" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="17"/>
+      <c r="F19" s="13"/>
       <c r="G19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H19" s="17" t="s">
+      <c r="H19" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="P19" s="17"/>
+      <c r="P19" s="13"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
@@ -1705,7 +1697,7 @@
       <c r="B20" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="18">
         <v>26</v>
       </c>
       <c r="D20" s="3">
@@ -1714,11 +1706,11 @@
       <c r="E20" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F20" s="17"/>
+      <c r="F20" s="13"/>
       <c r="G20" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H20" s="17" t="s">
+      <c r="H20" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I20" s="1"/>
@@ -1733,7 +1725,7 @@
       <c r="B21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="18">
         <v>23</v>
       </c>
       <c r="D21" s="3">
@@ -1745,7 +1737,7 @@
       <c r="G21" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H21" s="17" t="s">
+      <c r="H21" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I21" s="1"/>
@@ -1760,7 +1752,7 @@
       <c r="B22" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="18">
         <v>21</v>
       </c>
       <c r="D22" s="3">
@@ -1772,7 +1764,7 @@
       <c r="G22" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H22" s="17" t="s">
+      <c r="H22" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I22" s="1"/>
@@ -1787,7 +1779,7 @@
       <c r="B23" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="22">
+      <c r="C23" s="18">
         <v>24</v>
       </c>
       <c r="D23" s="3">
@@ -1799,7 +1791,7 @@
       <c r="G23" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H23" s="17" t="s">
+      <c r="H23" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I23" s="1"/>
@@ -1814,7 +1806,7 @@
       <c r="B24" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="18">
         <v>20</v>
       </c>
       <c r="D24" s="3">
@@ -1826,7 +1818,7 @@
       <c r="G24" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H24" s="17" t="s">
+      <c r="H24" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I24" s="1"/>
@@ -1841,7 +1833,7 @@
       <c r="B25" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="22">
+      <c r="C25" s="18">
         <v>27</v>
       </c>
       <c r="D25" s="3">
@@ -1853,7 +1845,7 @@
       <c r="G25" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H25" s="17" t="s">
+      <c r="H25" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I25" s="1"/>
@@ -1868,7 +1860,7 @@
       <c r="B26" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="22">
+      <c r="C26" s="18">
         <v>27</v>
       </c>
       <c r="D26" s="3">
@@ -1880,7 +1872,7 @@
       <c r="G26" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="H26" s="17" t="s">
+      <c r="H26" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I26" s="1"/>
@@ -1895,7 +1887,7 @@
       <c r="B27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="19">
         <v>28</v>
       </c>
       <c r="D27" s="3">
@@ -1907,7 +1899,7 @@
       <c r="G27" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H27" s="17" t="s">
+      <c r="H27" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I27" s="1"/>
@@ -1922,7 +1914,7 @@
       <c r="B28" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="22">
+      <c r="C28" s="18">
         <v>22</v>
       </c>
       <c r="D28" s="3">
@@ -1934,7 +1926,7 @@
       <c r="G28" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H28" s="17" t="s">
+      <c r="H28" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I28" s="1"/>
@@ -1949,7 +1941,7 @@
       <c r="B29" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C29" s="22">
+      <c r="C29" s="18">
         <v>29</v>
       </c>
       <c r="D29" s="3">
@@ -1961,7 +1953,7 @@
       <c r="G29" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H29" s="17" t="s">
+      <c r="H29" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I29" s="1"/>
@@ -1976,7 +1968,7 @@
       <c r="B30" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C30" s="22">
+      <c r="C30" s="18">
         <v>24</v>
       </c>
       <c r="D30" s="3">
@@ -1988,7 +1980,7 @@
       <c r="G30" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H30" s="17" t="s">
+      <c r="H30" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I30" s="1"/>
@@ -2003,7 +1995,7 @@
       <c r="B31" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="22">
+      <c r="C31" s="18">
         <v>24</v>
       </c>
       <c r="D31" s="3">
@@ -2015,7 +2007,7 @@
       <c r="G31" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H31" s="17" t="s">
+      <c r="H31" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I31" s="1"/>
@@ -2030,7 +2022,7 @@
       <c r="B32" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C32" s="22">
+      <c r="C32" s="18">
         <v>25</v>
       </c>
       <c r="D32" s="4">
@@ -2042,7 +2034,7 @@
       <c r="G32" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H32" s="17" t="s">
+      <c r="H32" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I32" s="5" t="s">
@@ -2059,7 +2051,7 @@
       <c r="B33" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C33" s="22">
+      <c r="C33" s="18">
         <v>26</v>
       </c>
       <c r="D33" s="3">
@@ -2071,7 +2063,7 @@
       <c r="G33" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H33" s="17" t="s">
+      <c r="H33" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I33" s="1"/>
@@ -2086,7 +2078,7 @@
       <c r="B34" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="22">
+      <c r="C34" s="18">
         <v>28</v>
       </c>
       <c r="D34" s="4">
@@ -2098,7 +2090,7 @@
       <c r="G34" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H34" s="17" t="s">
+      <c r="H34" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I34" s="5" t="s">
@@ -2115,7 +2107,7 @@
       <c r="B35" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C35" s="22">
+      <c r="C35" s="18">
         <v>24</v>
       </c>
       <c r="D35" s="4">
@@ -2127,7 +2119,7 @@
       <c r="G35" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H35" s="17" t="s">
+      <c r="H35" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I35" s="1"/>
@@ -2142,7 +2134,7 @@
       <c r="B36" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C36" s="22">
+      <c r="C36" s="18">
         <v>28</v>
       </c>
       <c r="D36" s="4">
@@ -2154,7 +2146,7 @@
       <c r="G36" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H36" s="17" t="s">
+      <c r="H36" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I36" s="1"/>
@@ -2169,7 +2161,7 @@
       <c r="B37" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C37" s="22">
+      <c r="C37" s="18">
         <v>29</v>
       </c>
       <c r="D37" s="3">
@@ -2181,7 +2173,7 @@
       <c r="G37" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H37" s="17" t="s">
+      <c r="H37" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I37" s="1"/>
@@ -2196,7 +2188,7 @@
       <c r="B38" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C38" s="22">
+      <c r="C38" s="18">
         <v>22</v>
       </c>
       <c r="D38" s="3">
@@ -2208,7 +2200,7 @@
       <c r="G38" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H38" s="17" t="s">
+      <c r="H38" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I38" s="1"/>
@@ -2223,7 +2215,7 @@
       <c r="B39" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C39" s="22">
+      <c r="C39" s="18">
         <v>27</v>
       </c>
       <c r="D39" s="3">
@@ -2235,7 +2227,7 @@
       <c r="G39" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H39" s="17" t="s">
+      <c r="H39" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I39" s="1"/>
@@ -2250,7 +2242,7 @@
       <c r="B40" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C40" s="22">
+      <c r="C40" s="18">
         <v>26</v>
       </c>
       <c r="D40" s="3">
@@ -2262,7 +2254,7 @@
       <c r="G40" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H40" s="17" t="s">
+      <c r="H40" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I40" s="1"/>
@@ -2271,26 +2263,25 @@
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A41" s="6">
+      <c r="A41" s="1">
         <v>327</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="C41" s="22">
+      <c r="C41" s="18">
         <v>29</v>
       </c>
-      <c r="D41" s="8">
+      <c r="D41" s="3">
         <v>35189</v>
       </c>
-      <c r="E41" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7" t="s">
+      <c r="E41" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H41" s="17" t="s">
+      <c r="H41" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I41" s="1"/>
@@ -2305,7 +2296,7 @@
       <c r="B42" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C42" s="22">
+      <c r="C42" s="18">
         <v>38</v>
       </c>
       <c r="D42" s="3">
@@ -2317,7 +2308,7 @@
       <c r="G42" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H42" s="17" t="s">
+      <c r="H42" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I42" s="1"/>
@@ -2332,7 +2323,7 @@
       <c r="B43" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C43" s="22">
+      <c r="C43" s="18">
         <v>39</v>
       </c>
       <c r="D43" s="3">
@@ -2344,7 +2335,7 @@
       <c r="G43" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H43" s="17" t="s">
+      <c r="H43" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I43" s="1"/>
@@ -2359,7 +2350,7 @@
       <c r="B44" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C44" s="22">
+      <c r="C44" s="18">
         <v>39</v>
       </c>
       <c r="D44" s="3">
@@ -2371,7 +2362,7 @@
       <c r="G44" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H44" s="17" t="s">
+      <c r="H44" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I44" s="1"/>
@@ -2386,7 +2377,7 @@
       <c r="B45" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C45" s="22">
+      <c r="C45" s="18">
         <v>39</v>
       </c>
       <c r="D45" s="3">
@@ -2398,7 +2389,7 @@
       <c r="G45" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="H45" s="17" t="s">
+      <c r="H45" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I45" s="1"/>
@@ -2413,7 +2404,7 @@
       <c r="B46" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C46" s="22">
+      <c r="C46" s="18">
         <v>37</v>
       </c>
       <c r="D46" s="3">
@@ -2425,7 +2416,7 @@
       <c r="G46" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H46" s="17" t="s">
+      <c r="H46" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I46" s="1"/>
@@ -2440,7 +2431,7 @@
       <c r="B47" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C47" s="22">
+      <c r="C47" s="18">
         <v>39</v>
       </c>
       <c r="D47" s="3">
@@ -2452,7 +2443,7 @@
       <c r="G47" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H47" s="17" t="s">
+      <c r="H47" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I47" s="1"/>
@@ -2467,7 +2458,7 @@
       <c r="B48" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C48" s="22">
+      <c r="C48" s="18">
         <v>32</v>
       </c>
       <c r="D48" s="4">
@@ -2479,7 +2470,7 @@
       <c r="G48" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H48" s="17" t="s">
+      <c r="H48" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I48" s="1"/>
@@ -2494,7 +2485,7 @@
       <c r="B49" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C49" s="22">
+      <c r="C49" s="18">
         <v>39</v>
       </c>
       <c r="D49" s="3">
@@ -2506,7 +2497,7 @@
       <c r="G49" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H49" s="17" t="s">
+      <c r="H49" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I49" s="1"/>
@@ -2521,7 +2512,7 @@
       <c r="B50" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C50" s="22">
+      <c r="C50" s="18">
         <v>33</v>
       </c>
       <c r="D50" s="3">
@@ -2533,7 +2524,7 @@
       <c r="G50" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H50" s="17" t="s">
+      <c r="H50" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I50" s="1"/>
@@ -2548,7 +2539,7 @@
       <c r="B51" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C51" s="22">
+      <c r="C51" s="18">
         <v>44</v>
       </c>
       <c r="D51" s="4">
@@ -2560,7 +2551,7 @@
       <c r="G51" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H51" s="17" t="s">
+      <c r="H51" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I51" s="1"/>
@@ -2575,7 +2566,7 @@
       <c r="B52" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C52" s="22">
+      <c r="C52" s="18">
         <v>37</v>
       </c>
       <c r="D52" s="4">
@@ -2587,7 +2578,7 @@
       <c r="G52" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H52" s="17" t="s">
+      <c r="H52" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I52" s="1"/>
@@ -2602,7 +2593,7 @@
       <c r="B53" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C53" s="23">
+      <c r="C53" s="19">
         <v>32</v>
       </c>
       <c r="D53" s="3">
@@ -2614,7 +2605,7 @@
       <c r="G53" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H53" s="17" t="s">
+      <c r="H53" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I53" s="1"/>
@@ -2629,7 +2620,7 @@
       <c r="B54" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C54" s="22">
+      <c r="C54" s="18">
         <v>35</v>
       </c>
       <c r="D54" s="3">
@@ -2641,7 +2632,7 @@
       <c r="G54" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H54" s="17" t="s">
+      <c r="H54" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I54" s="1"/>
@@ -2656,7 +2647,7 @@
       <c r="B55" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C55" s="22">
+      <c r="C55" s="18">
         <v>44</v>
       </c>
       <c r="D55" s="3">
@@ -2668,7 +2659,7 @@
       <c r="G55" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H55" s="17" t="s">
+      <c r="H55" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I55" s="1"/>
@@ -2683,7 +2674,7 @@
       <c r="B56" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C56" s="22">
+      <c r="C56" s="18">
         <v>35</v>
       </c>
       <c r="D56" s="4">
@@ -2695,7 +2686,7 @@
       <c r="G56" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H56" s="17" t="s">
+      <c r="H56" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I56" s="1"/>
@@ -2710,7 +2701,7 @@
       <c r="B57" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C57" s="22">
+      <c r="C57" s="18">
         <v>31</v>
       </c>
       <c r="D57" s="4">
@@ -2722,7 +2713,7 @@
       <c r="G57" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H57" s="17" t="s">
+      <c r="H57" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I57" s="1"/>
@@ -2737,7 +2728,7 @@
       <c r="B58" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C58" s="22">
+      <c r="C58" s="18">
         <v>33</v>
       </c>
       <c r="D58" s="3">
@@ -2749,7 +2740,7 @@
       <c r="G58" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H58" s="17" t="s">
+      <c r="H58" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I58" s="1"/>
@@ -2764,19 +2755,19 @@
       <c r="B59" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C59" s="24">
+      <c r="C59" s="20">
         <v>31</v>
       </c>
-      <c r="D59" s="9">
+      <c r="D59" s="6">
         <v>34441</v>
       </c>
-      <c r="E59" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G59" s="11" t="s">
+      <c r="E59" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G59" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="H59" s="17" t="s">
+      <c r="H59" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I59" s="1"/>
@@ -2791,7 +2782,7 @@
       <c r="B60" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C60" s="23">
+      <c r="C60" s="19">
         <v>36</v>
       </c>
       <c r="D60" s="3">
@@ -2803,7 +2794,7 @@
       <c r="G60" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H60" s="17" t="s">
+      <c r="H60" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I60" s="5" t="s">
@@ -2820,7 +2811,7 @@
       <c r="B61" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C61" s="22">
+      <c r="C61" s="18">
         <v>39</v>
       </c>
       <c r="D61" s="3">
@@ -2832,7 +2823,7 @@
       <c r="G61" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H61" s="17" t="s">
+      <c r="H61" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I61" s="1"/>
@@ -2847,7 +2838,7 @@
       <c r="B62" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C62" s="22">
+      <c r="C62" s="18">
         <v>40</v>
       </c>
       <c r="D62" s="4">
@@ -2859,7 +2850,7 @@
       <c r="G62" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H62" s="17" t="s">
+      <c r="H62" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I62" s="1"/>
@@ -2874,7 +2865,7 @@
       <c r="B63" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C63" s="22">
+      <c r="C63" s="18">
         <v>32</v>
       </c>
       <c r="D63" s="3">
@@ -2886,7 +2877,7 @@
       <c r="G63" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H63" s="17" t="s">
+      <c r="H63" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I63" s="1"/>
@@ -2901,7 +2892,7 @@
       <c r="B64" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C64" s="22">
+      <c r="C64" s="18">
         <v>43</v>
       </c>
       <c r="D64" s="4">
@@ -2913,7 +2904,7 @@
       <c r="G64" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H64" s="17" t="s">
+      <c r="H64" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I64" s="1"/>
@@ -2928,7 +2919,7 @@
       <c r="B65" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C65" s="22">
+      <c r="C65" s="18">
         <v>42</v>
       </c>
       <c r="D65" s="4">
@@ -2940,7 +2931,7 @@
       <c r="G65" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H65" s="17" t="s">
+      <c r="H65" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I65" s="1"/>
@@ -2955,7 +2946,7 @@
       <c r="B66" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C66" s="22">
+      <c r="C66" s="18">
         <v>43</v>
       </c>
       <c r="D66" s="3">
@@ -2967,7 +2958,7 @@
       <c r="G66" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H66" s="17" t="s">
+      <c r="H66" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I66" s="1"/>
@@ -2982,7 +2973,7 @@
       <c r="B67" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C67" s="22">
+      <c r="C67" s="18">
         <v>41</v>
       </c>
       <c r="D67" s="3">
@@ -2994,7 +2985,7 @@
       <c r="G67" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H67" s="17" t="s">
+      <c r="H67" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I67" s="1"/>
@@ -3009,7 +3000,7 @@
       <c r="B68" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C68" s="22">
+      <c r="C68" s="18">
         <v>39</v>
       </c>
       <c r="D68" s="3">
@@ -3021,7 +3012,7 @@
       <c r="G68" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H68" s="17" t="s">
+      <c r="H68" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I68" s="5" t="s">
@@ -3038,7 +3029,7 @@
       <c r="B69" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C69" s="22">
+      <c r="C69" s="18">
         <v>41</v>
       </c>
       <c r="D69" s="3">
@@ -3050,7 +3041,7 @@
       <c r="G69" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H69" s="17" t="s">
+      <c r="H69" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I69" s="1"/>
@@ -3065,7 +3056,7 @@
       <c r="B70" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C70" s="22">
+      <c r="C70" s="18">
         <v>40</v>
       </c>
       <c r="D70" s="4">
@@ -3077,7 +3068,7 @@
       <c r="G70" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H70" s="17" t="s">
+      <c r="H70" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I70" s="5" t="s">
@@ -3094,7 +3085,7 @@
       <c r="B71" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C71" s="22">
+      <c r="C71" s="18">
         <v>41</v>
       </c>
       <c r="D71" s="3">
@@ -3106,7 +3097,7 @@
       <c r="G71" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H71" s="17" t="s">
+      <c r="H71" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I71" s="1"/>
@@ -3121,7 +3112,7 @@
       <c r="B72" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C72" s="22">
+      <c r="C72" s="18">
         <v>37</v>
       </c>
       <c r="D72" s="4">
@@ -3133,7 +3124,7 @@
       <c r="G72" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H72" s="17" t="s">
+      <c r="H72" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I72" s="1"/>
@@ -3148,7 +3139,7 @@
       <c r="B73" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C73" s="22">
+      <c r="C73" s="18">
         <v>33</v>
       </c>
       <c r="D73" s="3">
@@ -3160,7 +3151,7 @@
       <c r="G73" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H73" s="17" t="s">
+      <c r="H73" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I73" s="1"/>
@@ -3175,7 +3166,7 @@
       <c r="B74" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C74" s="22">
+      <c r="C74" s="18">
         <v>42</v>
       </c>
       <c r="D74" s="3">
@@ -3187,7 +3178,7 @@
       <c r="G74" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H74" s="17" t="s">
+      <c r="H74" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I74" s="1"/>
@@ -3202,7 +3193,7 @@
       <c r="B75" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C75" s="22">
+      <c r="C75" s="18">
         <v>43</v>
       </c>
       <c r="D75" s="3">
@@ -3214,7 +3205,7 @@
       <c r="G75" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H75" s="17" t="s">
+      <c r="H75" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I75" s="1"/>
@@ -3229,7 +3220,7 @@
       <c r="B76" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C76" s="22">
+      <c r="C76" s="18">
         <v>37</v>
       </c>
       <c r="D76" s="3">
@@ -3241,7 +3232,7 @@
       <c r="G76" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H76" s="17" t="s">
+      <c r="H76" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I76" s="1"/>
@@ -3256,7 +3247,7 @@
       <c r="B77" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C77" s="22">
+      <c r="C77" s="18">
         <v>33</v>
       </c>
       <c r="D77" s="4">
@@ -3268,7 +3259,7 @@
       <c r="G77" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H77" s="17" t="s">
+      <c r="H77" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I77" s="1"/>
@@ -3283,7 +3274,7 @@
       <c r="B78" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C78" s="22">
+      <c r="C78" s="18">
         <v>32</v>
       </c>
       <c r="D78" s="3">
@@ -3295,7 +3286,7 @@
       <c r="G78" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="H78" s="17" t="s">
+      <c r="H78" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I78" s="1"/>
@@ -3310,7 +3301,7 @@
       <c r="B79" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C79" s="22">
+      <c r="C79" s="18">
         <v>44</v>
       </c>
       <c r="D79" s="3">
@@ -3322,7 +3313,7 @@
       <c r="G79" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="H79" s="17" t="s">
+      <c r="H79" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I79" s="1"/>
@@ -3337,7 +3328,7 @@
       <c r="B80" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C80" s="22">
+      <c r="C80" s="18">
         <v>40</v>
       </c>
       <c r="D80" s="4">
@@ -3349,7 +3340,7 @@
       <c r="G80" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H80" s="17" t="s">
+      <c r="H80" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I80" s="1"/>
@@ -3364,7 +3355,7 @@
       <c r="B81" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C81" s="22">
+      <c r="C81" s="18">
         <v>37</v>
       </c>
       <c r="D81" s="3">
@@ -3376,7 +3367,7 @@
       <c r="G81" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H81" s="17" t="s">
+      <c r="H81" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I81" s="1"/>
@@ -3391,7 +3382,7 @@
       <c r="B82" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C82" s="22">
+      <c r="C82" s="18">
         <v>30</v>
       </c>
       <c r="D82" s="3">
@@ -3403,7 +3394,7 @@
       <c r="G82" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H82" s="17" t="s">
+      <c r="H82" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I82" s="1"/>
@@ -3418,7 +3409,7 @@
       <c r="B83" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C83" s="22">
+      <c r="C83" s="18">
         <v>40</v>
       </c>
       <c r="D83" s="3">
@@ -3430,7 +3421,7 @@
       <c r="G83" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H83" s="17" t="s">
+      <c r="H83" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I83" s="1"/>
@@ -3445,7 +3436,7 @@
       <c r="B84" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C84" s="22">
+      <c r="C84" s="18">
         <v>37</v>
       </c>
       <c r="D84" s="4">
@@ -3457,7 +3448,7 @@
       <c r="G84" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H84" s="17" t="s">
+      <c r="H84" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I84" s="1"/>
@@ -3472,7 +3463,7 @@
       <c r="B85" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C85" s="22">
+      <c r="C85" s="18">
         <v>34</v>
       </c>
       <c r="D85" s="3">
@@ -3484,7 +3475,7 @@
       <c r="G85" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H85" s="17" t="s">
+      <c r="H85" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I85" s="1"/>
@@ -3499,7 +3490,7 @@
       <c r="B86" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C86" s="22">
+      <c r="C86" s="18">
         <v>33</v>
       </c>
       <c r="D86" s="3">
@@ -3511,7 +3502,7 @@
       <c r="G86" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H86" s="17" t="s">
+      <c r="H86" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I86" s="1"/>
@@ -3526,7 +3517,7 @@
       <c r="B87" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C87" s="22">
+      <c r="C87" s="18">
         <v>33</v>
       </c>
       <c r="D87" s="3">
@@ -3538,7 +3529,7 @@
       <c r="G87" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H87" s="17" t="s">
+      <c r="H87" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I87" s="1"/>
@@ -3553,7 +3544,7 @@
       <c r="B88" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C88" s="22">
+      <c r="C88" s="18">
         <v>42</v>
       </c>
       <c r="D88" s="3">
@@ -3565,7 +3556,7 @@
       <c r="G88" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H88" s="17" t="s">
+      <c r="H88" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I88" s="1"/>
@@ -3580,7 +3571,7 @@
       <c r="B89" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C89" s="22">
+      <c r="C89" s="18">
         <v>33</v>
       </c>
       <c r="D89" s="3">
@@ -3592,7 +3583,7 @@
       <c r="G89" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H89" s="17" t="s">
+      <c r="H89" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I89" s="1"/>
@@ -3607,7 +3598,7 @@
       <c r="B90" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C90" s="22">
+      <c r="C90" s="18">
         <v>33</v>
       </c>
       <c r="D90" s="3">
@@ -3619,7 +3610,7 @@
       <c r="G90" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="H90" s="17" t="s">
+      <c r="H90" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I90" s="1"/>
@@ -3634,7 +3625,7 @@
       <c r="B91" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C91" s="22">
+      <c r="C91" s="18">
         <v>39</v>
       </c>
       <c r="D91" s="4">
@@ -3646,7 +3637,7 @@
       <c r="G91" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H91" s="17" t="s">
+      <c r="H91" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I91" s="1"/>
@@ -3661,7 +3652,7 @@
       <c r="B92" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C92" s="22">
+      <c r="C92" s="18">
         <v>38</v>
       </c>
       <c r="D92" s="3">
@@ -3673,7 +3664,7 @@
       <c r="G92" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H92" s="17" t="s">
+      <c r="H92" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I92" s="1"/>
@@ -3688,7 +3679,7 @@
       <c r="B93" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C93" s="22">
+      <c r="C93" s="18">
         <v>40</v>
       </c>
       <c r="D93" s="3">
@@ -3700,7 +3691,7 @@
       <c r="G93" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H93" s="17" t="s">
+      <c r="H93" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I93" s="1"/>
@@ -3715,7 +3706,7 @@
       <c r="B94" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C94" s="22">
+      <c r="C94" s="18">
         <v>40</v>
       </c>
       <c r="D94" s="3">
@@ -3727,7 +3718,7 @@
       <c r="G94" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H94" s="17" t="s">
+      <c r="H94" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I94" s="1"/>
@@ -3742,7 +3733,7 @@
       <c r="B95" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C95" s="22">
+      <c r="C95" s="18">
         <v>37</v>
       </c>
       <c r="D95" s="3">
@@ -3754,7 +3745,7 @@
       <c r="G95" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H95" s="17" t="s">
+      <c r="H95" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I95" s="1"/>
@@ -3769,7 +3760,7 @@
       <c r="B96" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="C96" s="22">
+      <c r="C96" s="18">
         <v>37</v>
       </c>
       <c r="D96" s="3">
@@ -3781,7 +3772,7 @@
       <c r="G96" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H96" s="17" t="s">
+      <c r="H96" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I96" s="1"/>
@@ -3796,7 +3787,7 @@
       <c r="B97" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="C97" s="22">
+      <c r="C97" s="18">
         <v>33</v>
       </c>
       <c r="D97" s="3">
@@ -3808,7 +3799,7 @@
       <c r="G97" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H97" s="17" t="s">
+      <c r="H97" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I97" s="1"/>
@@ -3823,7 +3814,7 @@
       <c r="B98" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C98" s="22">
+      <c r="C98" s="18">
         <v>35</v>
       </c>
       <c r="D98" s="3">
@@ -3835,7 +3826,7 @@
       <c r="G98" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H98" s="17" t="s">
+      <c r="H98" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I98" s="1"/>
@@ -3844,29 +3835,28 @@
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A99" s="6">
+      <c r="A99" s="1">
         <v>360</v>
       </c>
-      <c r="B99" s="7" t="s">
+      <c r="B99" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C99" s="22">
+      <c r="C99" s="18">
         <v>44</v>
       </c>
-      <c r="D99" s="8">
+      <c r="D99" s="3">
         <v>29888</v>
       </c>
-      <c r="E99" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="F99" s="7"/>
-      <c r="G99" s="7" t="s">
+      <c r="E99" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G99" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H99" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="I99" s="6"/>
+      <c r="H99" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I99" s="1"/>
       <c r="J99" s="2" t="s">
         <v>207</v>
       </c>
@@ -3878,7 +3868,7 @@
       <c r="B100" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C100" s="22">
+      <c r="C100" s="18">
         <v>31</v>
       </c>
       <c r="D100" s="4">
@@ -3890,7 +3880,7 @@
       <c r="G100" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H100" s="17" t="s">
+      <c r="H100" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I100" s="1"/>
@@ -3905,7 +3895,7 @@
       <c r="B101" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C101" s="22">
+      <c r="C101" s="18">
         <v>38</v>
       </c>
       <c r="D101" s="4">
@@ -3917,7 +3907,7 @@
       <c r="G101" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H101" s="17" t="s">
+      <c r="H101" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I101" s="1"/>
@@ -3932,7 +3922,7 @@
       <c r="B102" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C102" s="22">
+      <c r="C102" s="18">
         <v>33</v>
       </c>
       <c r="D102" s="3">
@@ -3944,7 +3934,7 @@
       <c r="G102" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H102" s="17" t="s">
+      <c r="H102" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I102" s="1"/>
@@ -3959,7 +3949,7 @@
       <c r="B103" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C103" s="23">
+      <c r="C103" s="19">
         <v>42</v>
       </c>
       <c r="D103" s="3">
@@ -3971,7 +3961,7 @@
       <c r="G103" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="H103" s="17" t="s">
+      <c r="H103" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I103" s="5" t="s">
@@ -3988,7 +3978,7 @@
       <c r="B104" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="C104" s="22">
+      <c r="C104" s="18">
         <v>42</v>
       </c>
       <c r="D104" s="4">
@@ -4000,7 +3990,7 @@
       <c r="G104" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H104" s="17" t="s">
+      <c r="H104" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I104" s="1"/>
@@ -4015,7 +4005,7 @@
       <c r="B105" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C105" s="22">
+      <c r="C105" s="18">
         <v>37</v>
       </c>
       <c r="D105" s="3">
@@ -4027,7 +4017,7 @@
       <c r="G105" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H105" s="17" t="s">
+      <c r="H105" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I105" s="1"/>
@@ -4042,7 +4032,7 @@
       <c r="B106" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C106" s="22">
+      <c r="C106" s="18">
         <v>34</v>
       </c>
       <c r="D106" s="3">
@@ -4054,7 +4044,7 @@
       <c r="G106" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H106" s="17" t="s">
+      <c r="H106" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I106" s="1"/>
@@ -4069,7 +4059,7 @@
       <c r="B107" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C107" s="22">
+      <c r="C107" s="18">
         <v>43</v>
       </c>
       <c r="D107" s="3">
@@ -4081,7 +4071,7 @@
       <c r="G107" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H107" s="17" t="s">
+      <c r="H107" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I107" s="1"/>
@@ -4096,7 +4086,7 @@
       <c r="B108" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C108" s="22">
+      <c r="C108" s="18">
         <v>44</v>
       </c>
       <c r="D108" s="3">
@@ -4108,7 +4098,7 @@
       <c r="G108" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H108" s="17" t="s">
+      <c r="H108" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I108" s="1"/>
@@ -4123,7 +4113,7 @@
       <c r="B109" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="C109" s="22">
+      <c r="C109" s="18">
         <v>43</v>
       </c>
       <c r="D109" s="3">
@@ -4135,7 +4125,7 @@
       <c r="G109" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H109" s="17" t="s">
+      <c r="H109" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I109" s="1"/>
@@ -4150,7 +4140,7 @@
       <c r="B110" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="C110" s="22">
+      <c r="C110" s="18">
         <v>44</v>
       </c>
       <c r="D110" s="3">
@@ -4162,7 +4152,7 @@
       <c r="G110" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H110" s="17" t="s">
+      <c r="H110" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I110" s="1"/>
@@ -4177,7 +4167,7 @@
       <c r="B111" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="C111" s="22">
+      <c r="C111" s="18">
         <v>40</v>
       </c>
       <c r="D111" s="4">
@@ -4189,7 +4179,7 @@
       <c r="G111" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H111" s="17" t="s">
+      <c r="H111" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I111" s="1"/>
@@ -4204,7 +4194,7 @@
       <c r="B112" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C112" s="22">
+      <c r="C112" s="18">
         <v>39</v>
       </c>
       <c r="D112" s="3">
@@ -4216,7 +4206,7 @@
       <c r="G112" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H112" s="17" t="s">
+      <c r="H112" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I112" s="1"/>
@@ -4231,7 +4221,7 @@
       <c r="B113" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C113" s="22">
+      <c r="C113" s="18">
         <v>39</v>
       </c>
       <c r="D113" s="3">
@@ -4243,7 +4233,7 @@
       <c r="G113" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H113" s="17" t="s">
+      <c r="H113" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I113" s="1"/>
@@ -4258,7 +4248,7 @@
       <c r="B114" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C114" s="22">
+      <c r="C114" s="18">
         <v>33</v>
       </c>
       <c r="D114" s="3">
@@ -4270,7 +4260,7 @@
       <c r="G114" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H114" s="17" t="s">
+      <c r="H114" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I114" s="1"/>
@@ -4285,7 +4275,7 @@
       <c r="B115" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C115" s="22">
+      <c r="C115" s="18">
         <v>33</v>
       </c>
       <c r="D115" s="3">
@@ -4297,7 +4287,7 @@
       <c r="G115" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H115" s="17" t="s">
+      <c r="H115" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I115" s="1"/>
@@ -4312,7 +4302,7 @@
       <c r="B116" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C116" s="22">
+      <c r="C116" s="18">
         <v>42</v>
       </c>
       <c r="D116" s="3">
@@ -4324,7 +4314,7 @@
       <c r="G116" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H116" s="17" t="s">
+      <c r="H116" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I116" s="1"/>
@@ -4339,7 +4329,7 @@
       <c r="B117" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C117" s="22">
+      <c r="C117" s="18">
         <v>39</v>
       </c>
       <c r="D117" s="4">
@@ -4351,7 +4341,7 @@
       <c r="G117" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H117" s="17" t="s">
+      <c r="H117" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I117" s="1"/>
@@ -4366,7 +4356,7 @@
       <c r="B118" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C118" s="22">
+      <c r="C118" s="18">
         <v>36</v>
       </c>
       <c r="D118" s="3">
@@ -4378,7 +4368,7 @@
       <c r="G118" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H118" s="17" t="s">
+      <c r="H118" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I118" s="1"/>
@@ -4393,7 +4383,7 @@
       <c r="B119" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C119" s="22">
+      <c r="C119" s="18">
         <v>44</v>
       </c>
       <c r="D119" s="3">
@@ -4405,7 +4395,7 @@
       <c r="G119" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H119" s="17" t="s">
+      <c r="H119" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I119" s="1"/>
@@ -4420,7 +4410,7 @@
       <c r="B120" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C120" s="22">
+      <c r="C120" s="18">
         <v>39</v>
       </c>
       <c r="D120" s="4">
@@ -4432,7 +4422,7 @@
       <c r="G120" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H120" s="17" t="s">
+      <c r="H120" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I120" s="1"/>
@@ -4447,7 +4437,7 @@
       <c r="B121" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C121" s="23">
+      <c r="C121" s="19">
         <v>31</v>
       </c>
       <c r="D121" s="3">
@@ -4459,7 +4449,7 @@
       <c r="G121" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H121" s="17" t="s">
+      <c r="H121" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I121" s="1"/>
@@ -4468,28 +4458,28 @@
       </c>
     </row>
     <row r="122" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A122" s="18">
+      <c r="A122" s="14">
         <v>383</v>
       </c>
-      <c r="B122" s="13" t="s">
+      <c r="B122" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="C122" s="23">
+      <c r="C122" s="19">
         <v>33</v>
       </c>
-      <c r="D122" s="19">
+      <c r="D122" s="15">
         <v>34141</v>
       </c>
-      <c r="E122" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="G122" s="21" t="s">
+      <c r="E122" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="G122" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="H122" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="I122" s="18"/>
+      <c r="H122" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I122" s="14"/>
       <c r="J122" s="2" t="s">
         <v>207</v>
       </c>
@@ -4501,7 +4491,7 @@
       <c r="B123" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C123" s="23">
+      <c r="C123" s="19">
         <v>34</v>
       </c>
       <c r="D123" s="3">
@@ -4513,7 +4503,7 @@
       <c r="G123" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="H123" s="17" t="s">
+      <c r="H123" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I123" s="1"/>
@@ -4528,7 +4518,7 @@
       <c r="B124" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="C124" s="23">
+      <c r="C124" s="19">
         <v>38</v>
       </c>
       <c r="D124" s="3">
@@ -4540,7 +4530,7 @@
       <c r="G124" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H124" s="17" t="s">
+      <c r="H124" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J124" s="2" t="s">
@@ -4554,7 +4544,7 @@
       <c r="B125" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="C125" s="23">
+      <c r="C125" s="19">
         <v>46</v>
       </c>
       <c r="D125" s="3">
@@ -4566,7 +4556,7 @@
       <c r="G125" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H125" s="17" t="s">
+      <c r="H125" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I125" s="1"/>
@@ -4581,7 +4571,7 @@
       <c r="B126" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="C126" s="22">
+      <c r="C126" s="18">
         <v>47</v>
       </c>
       <c r="D126" s="3">
@@ -4593,7 +4583,7 @@
       <c r="G126" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H126" s="17" t="s">
+      <c r="H126" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I126" s="1"/>
@@ -4608,7 +4598,7 @@
       <c r="B127" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C127" s="22">
+      <c r="C127" s="18">
         <v>57</v>
       </c>
       <c r="D127" s="3">
@@ -4620,7 +4610,7 @@
       <c r="G127" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H127" s="17" t="s">
+      <c r="H127" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I127" s="1"/>
@@ -4635,7 +4625,7 @@
       <c r="B128" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C128" s="22">
+      <c r="C128" s="18">
         <v>45</v>
       </c>
       <c r="D128" s="3">
@@ -4647,7 +4637,7 @@
       <c r="G128" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H128" s="17" t="s">
+      <c r="H128" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I128" s="5" t="s">
@@ -4664,7 +4654,7 @@
       <c r="B129" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C129" s="22">
+      <c r="C129" s="18">
         <v>46</v>
       </c>
       <c r="D129" s="3">
@@ -4676,7 +4666,7 @@
       <c r="G129" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="H129" s="17" t="s">
+      <c r="H129" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I129" s="1"/>
@@ -4691,7 +4681,7 @@
       <c r="B130" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="C130" s="22">
+      <c r="C130" s="18">
         <v>46</v>
       </c>
       <c r="D130" s="3">
@@ -4703,7 +4693,7 @@
       <c r="G130" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H130" s="17" t="s">
+      <c r="H130" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I130" s="1"/>
@@ -4718,7 +4708,7 @@
       <c r="B131" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C131" s="22">
+      <c r="C131" s="18">
         <v>49</v>
       </c>
       <c r="D131" s="3">
@@ -4730,7 +4720,7 @@
       <c r="G131" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H131" s="17" t="s">
+      <c r="H131" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I131" s="1"/>
@@ -4745,7 +4735,7 @@
       <c r="B132" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C132" s="22">
+      <c r="C132" s="18">
         <v>49</v>
       </c>
       <c r="D132" s="3">
@@ -4757,7 +4747,7 @@
       <c r="G132" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H132" s="17" t="s">
+      <c r="H132" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I132" s="1"/>
@@ -4772,7 +4762,7 @@
       <c r="B133" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C133" s="22">
+      <c r="C133" s="18">
         <v>45</v>
       </c>
       <c r="D133" s="3">
@@ -4784,7 +4774,7 @@
       <c r="G133" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H133" s="17" t="s">
+      <c r="H133" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I133" s="1"/>
@@ -4799,7 +4789,7 @@
       <c r="B134" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="C134" s="22">
+      <c r="C134" s="18">
         <v>49</v>
       </c>
       <c r="D134" s="3">
@@ -4811,7 +4801,7 @@
       <c r="G134" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H134" s="17" t="s">
+      <c r="H134" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I134" s="1"/>
@@ -4826,7 +4816,7 @@
       <c r="B135" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C135" s="22">
+      <c r="C135" s="18">
         <v>50</v>
       </c>
       <c r="D135" s="3">
@@ -4838,7 +4828,7 @@
       <c r="G135" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H135" s="17" t="s">
+      <c r="H135" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I135" s="1"/>
@@ -4853,7 +4843,7 @@
       <c r="B136" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C136" s="22">
+      <c r="C136" s="18">
         <v>49</v>
       </c>
       <c r="D136" s="3">
@@ -4865,7 +4855,7 @@
       <c r="G136" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="H136" s="17" t="s">
+      <c r="H136" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I136" s="1"/>
@@ -4880,7 +4870,7 @@
       <c r="B137" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="C137" s="22">
+      <c r="C137" s="18">
         <v>45</v>
       </c>
       <c r="D137" s="3">
@@ -4892,7 +4882,7 @@
       <c r="G137" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H137" s="17" t="s">
+      <c r="H137" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I137" s="1"/>
@@ -4907,7 +4897,7 @@
       <c r="B138" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C138" s="22">
+      <c r="C138" s="18">
         <v>51</v>
       </c>
       <c r="D138" s="3">
@@ -4919,7 +4909,7 @@
       <c r="G138" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H138" s="17" t="s">
+      <c r="H138" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I138" s="5" t="s">
@@ -4936,7 +4926,7 @@
       <c r="B139" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C139" s="22">
+      <c r="C139" s="18">
         <v>48</v>
       </c>
       <c r="D139" s="3">
@@ -4948,7 +4938,7 @@
       <c r="G139" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="H139" s="17" t="s">
+      <c r="H139" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I139" s="1"/>
@@ -4963,7 +4953,7 @@
       <c r="B140" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C140" s="22">
+      <c r="C140" s="18">
         <v>46</v>
       </c>
       <c r="D140" s="3">
@@ -4975,7 +4965,7 @@
       <c r="G140" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H140" s="17" t="s">
+      <c r="H140" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I140" s="1"/>
@@ -4990,7 +4980,7 @@
       <c r="B141" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="C141" s="22">
+      <c r="C141" s="18">
         <v>59</v>
       </c>
       <c r="D141" s="3">
@@ -5002,7 +4992,7 @@
       <c r="G141" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H141" s="17" t="s">
+      <c r="H141" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I141" s="1"/>
@@ -5017,7 +5007,7 @@
       <c r="B142" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C142" s="22">
+      <c r="C142" s="18">
         <v>46</v>
       </c>
       <c r="D142" s="3">
@@ -5029,7 +5019,7 @@
       <c r="G142" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H142" s="17" t="s">
+      <c r="H142" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I142" s="1"/>
@@ -5044,7 +5034,7 @@
       <c r="B143" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C143" s="23">
+      <c r="C143" s="19">
         <v>54</v>
       </c>
       <c r="D143" s="3">
@@ -5056,7 +5046,7 @@
       <c r="G143" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="H143" s="17" t="s">
+      <c r="H143" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I143" s="1"/>
@@ -5071,7 +5061,7 @@
       <c r="B144" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C144" s="22">
+      <c r="C144" s="18">
         <v>46</v>
       </c>
       <c r="D144" s="3">
@@ -5083,7 +5073,7 @@
       <c r="G144" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="H144" s="17" t="s">
+      <c r="H144" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I144" s="1"/>
@@ -5098,7 +5088,7 @@
       <c r="B145" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C145" s="22">
+      <c r="C145" s="18">
         <v>48</v>
       </c>
       <c r="D145" s="3">
@@ -5110,7 +5100,7 @@
       <c r="G145" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H145" s="17" t="s">
+      <c r="H145" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I145" s="1"/>
@@ -5125,7 +5115,7 @@
       <c r="B146" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C146" s="22">
+      <c r="C146" s="18">
         <v>53</v>
       </c>
       <c r="D146" s="3">
@@ -5137,7 +5127,7 @@
       <c r="G146" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H146" s="17" t="s">
+      <c r="H146" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I146" s="1"/>
@@ -5152,7 +5142,7 @@
       <c r="B147" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C147" s="22">
+      <c r="C147" s="18">
         <v>49</v>
       </c>
       <c r="D147" s="3">
@@ -5164,7 +5154,7 @@
       <c r="G147" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="H147" s="17" t="s">
+      <c r="H147" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I147" s="1"/>
@@ -5179,7 +5169,7 @@
       <c r="B148" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="C148" s="22">
+      <c r="C148" s="18">
         <v>53</v>
       </c>
       <c r="D148" s="4">
@@ -5191,7 +5181,7 @@
       <c r="G148" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H148" s="17" t="s">
+      <c r="H148" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I148" s="1"/>
@@ -5206,7 +5196,7 @@
       <c r="B149" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C149" s="22">
+      <c r="C149" s="18">
         <v>52</v>
       </c>
       <c r="D149" s="3">
@@ -5218,7 +5208,7 @@
       <c r="G149" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H149" s="17" t="s">
+      <c r="H149" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I149" s="1"/>
@@ -5233,7 +5223,7 @@
       <c r="B150" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="C150" s="22">
+      <c r="C150" s="18">
         <v>59</v>
       </c>
       <c r="D150" s="3">
@@ -5245,7 +5235,7 @@
       <c r="G150" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H150" s="17" t="s">
+      <c r="H150" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I150" s="1"/>
@@ -5260,7 +5250,7 @@
       <c r="B151" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C151" s="22">
+      <c r="C151" s="18">
         <v>52</v>
       </c>
       <c r="D151" s="3">
@@ -5272,7 +5262,7 @@
       <c r="G151" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H151" s="17" t="s">
+      <c r="H151" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I151" s="1"/>
@@ -5287,7 +5277,7 @@
       <c r="B152" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="C152" s="22">
+      <c r="C152" s="18">
         <v>59</v>
       </c>
       <c r="D152" s="3">
@@ -5299,7 +5289,7 @@
       <c r="G152" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H152" s="17" t="s">
+      <c r="H152" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I152" s="1"/>
@@ -5314,7 +5304,7 @@
       <c r="B153" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C153" s="22">
+      <c r="C153" s="18">
         <v>51</v>
       </c>
       <c r="D153" s="3">
@@ -5326,7 +5316,7 @@
       <c r="G153" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="H153" s="17" t="s">
+      <c r="H153" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I153" s="1"/>
@@ -5341,7 +5331,7 @@
       <c r="B154" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="C154" s="23">
+      <c r="C154" s="19">
         <v>47</v>
       </c>
       <c r="D154" s="3">
@@ -5353,7 +5343,7 @@
       <c r="G154" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="H154" s="17" t="s">
+      <c r="H154" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I154" s="5" t="s">
@@ -5370,7 +5360,7 @@
       <c r="B155" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="C155" s="22">
+      <c r="C155" s="18">
         <v>49</v>
       </c>
       <c r="D155" s="3">
@@ -5382,7 +5372,7 @@
       <c r="G155" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H155" s="17" t="s">
+      <c r="H155" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I155" s="1"/>
@@ -5397,7 +5387,7 @@
       <c r="B156" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="C156" s="22">
+      <c r="C156" s="18">
         <v>56</v>
       </c>
       <c r="D156" s="4">
@@ -5409,7 +5399,7 @@
       <c r="G156" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H156" s="17" t="s">
+      <c r="H156" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I156" s="1"/>
@@ -5424,7 +5414,7 @@
       <c r="B157" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C157" s="22">
+      <c r="C157" s="18">
         <v>45</v>
       </c>
       <c r="D157" s="3">
@@ -5436,7 +5426,7 @@
       <c r="G157" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H157" s="17" t="s">
+      <c r="H157" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I157" s="1"/>
@@ -5451,7 +5441,7 @@
       <c r="B158" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="C158" s="22">
+      <c r="C158" s="18">
         <v>45</v>
       </c>
       <c r="D158" s="3">
@@ -5463,7 +5453,7 @@
       <c r="G158" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H158" s="17" t="s">
+      <c r="H158" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I158" s="1"/>
@@ -5478,7 +5468,7 @@
       <c r="B159" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="C159" s="22">
+      <c r="C159" s="18">
         <v>49</v>
       </c>
       <c r="D159" s="3">
@@ -5490,7 +5480,7 @@
       <c r="G159" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H159" s="17" t="s">
+      <c r="H159" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I159" s="1"/>
@@ -5505,7 +5495,7 @@
       <c r="B160" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="C160" s="22">
+      <c r="C160" s="18">
         <v>45</v>
       </c>
       <c r="D160" s="4">
@@ -5517,7 +5507,7 @@
       <c r="G160" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H160" s="17" t="s">
+      <c r="H160" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I160" s="1"/>
@@ -5532,7 +5522,7 @@
       <c r="B161" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C161" s="22">
+      <c r="C161" s="18">
         <v>58</v>
       </c>
       <c r="D161" s="3">
@@ -5544,7 +5534,7 @@
       <c r="G161" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H161" s="17" t="s">
+      <c r="H161" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I161" s="1"/>
@@ -5559,7 +5549,7 @@
       <c r="B162" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C162" s="22">
+      <c r="C162" s="18">
         <v>55</v>
       </c>
       <c r="D162" s="4">
@@ -5571,7 +5561,7 @@
       <c r="G162" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H162" s="17" t="s">
+      <c r="H162" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I162" s="1"/>
@@ -5586,7 +5576,7 @@
       <c r="B163" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C163" s="22">
+      <c r="C163" s="18">
         <v>68</v>
       </c>
       <c r="D163" s="3">
@@ -5598,7 +5588,7 @@
       <c r="G163" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H163" s="17" t="s">
+      <c r="H163" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J163" s="2" t="s">
@@ -5612,7 +5602,7 @@
       <c r="B164" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C164" s="22">
+      <c r="C164" s="18">
         <v>60</v>
       </c>
       <c r="D164" s="4">
@@ -5624,7 +5614,7 @@
       <c r="G164" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H164" s="17" t="s">
+      <c r="H164" s="13" t="s">
         <v>10</v>
       </c>
       <c r="I164" s="5" t="s">
@@ -5641,7 +5631,7 @@
       <c r="B165" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C165" s="22">
+      <c r="C165" s="18">
         <v>63</v>
       </c>
       <c r="D165" s="3">
@@ -5653,7 +5643,7 @@
       <c r="G165" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H165" s="17" t="s">
+      <c r="H165" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J165" s="2" t="s">
@@ -5667,7 +5657,7 @@
       <c r="B166" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="C166" s="22">
+      <c r="C166" s="18">
         <v>60</v>
       </c>
       <c r="D166" s="3">
@@ -5679,7 +5669,7 @@
       <c r="G166" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H166" s="17" t="s">
+      <c r="H166" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J166" s="2" t="s">
@@ -5693,7 +5683,7 @@
       <c r="B167" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C167" s="22">
+      <c r="C167" s="18">
         <v>61</v>
       </c>
       <c r="D167" s="3">
@@ -5705,7 +5695,7 @@
       <c r="G167" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H167" s="17" t="s">
+      <c r="H167" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J167" s="2" t="s">
@@ -5719,7 +5709,7 @@
       <c r="B168" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C168" s="22">
+      <c r="C168" s="18">
         <v>62</v>
       </c>
       <c r="D168" s="3">
@@ -5731,7 +5721,7 @@
       <c r="G168" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H168" s="17" t="s">
+      <c r="H168" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J168" s="2" t="s">
@@ -5745,7 +5735,7 @@
       <c r="B169" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="C169" s="22">
+      <c r="C169" s="18">
         <v>60</v>
       </c>
       <c r="D169" s="3">
@@ -5757,7 +5747,7 @@
       <c r="G169" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H169" s="17" t="s">
+      <c r="H169" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J169" s="2" t="s">
@@ -5771,7 +5761,7 @@
       <c r="B170" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="C170" s="22">
+      <c r="C170" s="18">
         <v>60</v>
       </c>
       <c r="D170" s="3">
@@ -5783,7 +5773,7 @@
       <c r="G170" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="H170" s="17" t="s">
+      <c r="H170" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J170" s="2" t="s">
@@ -5797,7 +5787,7 @@
       <c r="B171" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="C171" s="22">
+      <c r="C171" s="18">
         <v>60</v>
       </c>
       <c r="D171" s="4">
@@ -5809,7 +5799,7 @@
       <c r="G171" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H171" s="17" t="s">
+      <c r="H171" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J171" s="2" t="s">
@@ -5823,7 +5813,7 @@
       <c r="B172" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="C172" s="23">
+      <c r="C172" s="19">
         <v>61</v>
       </c>
       <c r="D172" s="3">
@@ -5835,7 +5825,7 @@
       <c r="G172" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="H172" s="17" t="s">
+      <c r="H172" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J172" s="2" t="s">
@@ -5846,10 +5836,10 @@
       <c r="A173" s="1">
         <v>70</v>
       </c>
-      <c r="B173" s="14" t="s">
+      <c r="B173" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="C173" s="23">
+      <c r="C173" s="19">
         <v>63</v>
       </c>
       <c r="D173" s="3">
@@ -5861,7 +5851,7 @@
       <c r="G173" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="H173" s="17" t="s">
+      <c r="H173" s="13" t="s">
         <v>10</v>
       </c>
       <c r="J173" s="2" t="s">

</xml_diff>